<commit_message>
added datasheets and Bestellliste
</commit_message>
<xml_diff>
--- a/Komponenten und Auslegung/Bestellliste.xlsx
+++ b/Komponenten und Auslegung/Bestellliste.xlsx
@@ -5,27 +5,38 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxec\Documents\Studium\4. Semester\Elektronische Produktentwicklung I\AAAA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxec\Documents\Studium\4. Semester\Elektronische Produktentwicklung I\Komponenten und Auslegung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B38E223F-A497-4FA9-82C2-1C89A36E98A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A91B873-11FE-4FBD-BFE2-D9C288D8FEF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="41">
   <si>
     <t>Type</t>
   </si>
@@ -118,13 +129,46 @@
   </si>
   <si>
     <t>PCB-Komponenten:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mouser.at/ProductDetail/STMicroelectronics/STM32H7A3RIT6?qs=xZ%2FP%252Ba9zWqZAEQXxnLVEdg%3D%3D&amp;srsltid=AfmBOoouvnp0ZWZPSWktYUAhuhxXh0gnSv1AlPj8DEV16z0aPM-bQKXm </t>
+  </si>
+  <si>
+    <t>STMicroelectronics STM32H7A3RIT6</t>
+  </si>
+  <si>
+    <t>µC</t>
+  </si>
+  <si>
+    <t>ungefähre Kosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mouser.at/ProductDetail/Espressif-Systems/ESP8266EX?qs=chTDxNqvsynorwcu2ADV3g%3D%3D </t>
+  </si>
+  <si>
+    <t>Wi-Fi Chip</t>
+  </si>
+  <si>
+    <t>Espressif Systems ESP8266EX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mouser.at/ProductDetail/FTDI/FT2232HL-REEL?qs=D1%2FPMqvA100v7FHcEx164g%3D%3D </t>
+  </si>
+  <si>
+    <t>USB-UART</t>
+  </si>
+  <si>
+    <t>FTDI FT2232HL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -158,6 +202,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -167,7 +226,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -375,12 +434,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -404,10 +477,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Währung" xfId="2" builtinId="4"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -685,22 +765,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:E40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A2:F41"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.19921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="86.3984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="6.19921875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="255.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="86.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B2" s="22" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -714,10 +795,13 @@
         <v>5</v>
       </c>
       <c r="E4" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>22</v>
       </c>
@@ -730,9 +814,12 @@
       <c r="D5" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="8"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E5" s="24">
+        <v>0</v>
+      </c>
+      <c r="F5" s="8"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -745,9 +832,12 @@
       <c r="D6" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="8"/>
-    </row>
-    <row r="7" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="E6" s="24">
+        <v>0</v>
+      </c>
+      <c r="F6" s="8"/>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
         <v>27</v>
       </c>
@@ -760,11 +850,14 @@
       <c r="D7" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="25">
+        <v>40</v>
+      </c>
+      <c r="F7" s="17" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
         <v>9</v>
       </c>
@@ -777,11 +870,14 @@
       <c r="D8" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="21" t="s">
+      <c r="E8" s="26">
+        <v>60</v>
+      </c>
+      <c r="F8" s="21" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
@@ -794,11 +890,14 @@
       <c r="D9" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="24">
+        <v>20</v>
+      </c>
+      <c r="F9" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>14</v>
       </c>
@@ -811,11 +910,14 @@
       <c r="D10" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="24">
+        <v>80</v>
+      </c>
+      <c r="F10" s="9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>21</v>
       </c>
@@ -828,11 +930,14 @@
       <c r="D11" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="24">
+        <v>20</v>
+      </c>
+      <c r="F11" s="9" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>15</v>
       </c>
@@ -845,17 +950,20 @@
       <c r="D12" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="27">
+        <v>18</v>
+      </c>
+      <c r="F12" s="10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B14" s="22" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>0</v>
       </c>
@@ -868,186 +976,257 @@
       <c r="D16" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="7"/>
+      <c r="F16" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A17" s="2"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="8"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A18" s="2"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="8"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A19" s="2"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="8"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="5">
+        <v>1</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="24">
+        <v>14.5</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="5">
+        <v>1</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="24">
+        <v>2</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="5">
+        <v>1</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" s="24">
+        <v>5</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="12"/>
       <c r="C20" s="5"/>
       <c r="D20" s="12"/>
-      <c r="E20" s="8"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E20" s="24"/>
+      <c r="F20" s="8"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="12"/>
       <c r="C21" s="5"/>
       <c r="D21" s="12"/>
-      <c r="E21" s="8"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E21" s="24"/>
+      <c r="F21" s="8"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="12"/>
       <c r="C22" s="5"/>
       <c r="D22" s="12"/>
-      <c r="E22" s="8"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E22" s="24"/>
+      <c r="F22" s="8"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="12"/>
       <c r="C23" s="5"/>
       <c r="D23" s="12"/>
-      <c r="E23" s="8"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E23" s="24"/>
+      <c r="F23" s="8"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="12"/>
       <c r="C24" s="5"/>
       <c r="D24" s="12"/>
-      <c r="E24" s="8"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E24" s="24"/>
+      <c r="F24" s="8"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="12"/>
       <c r="C25" s="5"/>
       <c r="D25" s="12"/>
-      <c r="E25" s="8"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E25" s="24"/>
+      <c r="F25" s="8"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="12"/>
       <c r="C26" s="5"/>
       <c r="D26" s="12"/>
-      <c r="E26" s="8"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E26" s="24"/>
+      <c r="F26" s="8"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="12"/>
       <c r="C27" s="5"/>
       <c r="D27" s="12"/>
-      <c r="E27" s="8"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E27" s="24"/>
+      <c r="F27" s="8"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="12"/>
       <c r="C28" s="5"/>
       <c r="D28" s="12"/>
-      <c r="E28" s="8"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E28" s="24"/>
+      <c r="F28" s="8"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="12"/>
       <c r="C29" s="5"/>
       <c r="D29" s="12"/>
-      <c r="E29" s="8"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E29" s="24"/>
+      <c r="F29" s="8"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="12"/>
       <c r="C30" s="5"/>
       <c r="D30" s="12"/>
-      <c r="E30" s="8"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E30" s="24"/>
+      <c r="F30" s="8"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="12"/>
       <c r="C31" s="5"/>
       <c r="D31" s="12"/>
-      <c r="E31" s="8"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E31" s="24"/>
+      <c r="F31" s="8"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="12"/>
       <c r="C32" s="5"/>
       <c r="D32" s="12"/>
-      <c r="E32" s="8"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E32" s="24"/>
+      <c r="F32" s="8"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="12"/>
       <c r="C33" s="5"/>
       <c r="D33" s="12"/>
-      <c r="E33" s="8"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E33" s="24"/>
+      <c r="F33" s="8"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="12"/>
       <c r="C34" s="5"/>
       <c r="D34" s="12"/>
-      <c r="E34" s="8"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E34" s="24"/>
+      <c r="F34" s="8"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="12"/>
       <c r="C35" s="5"/>
       <c r="D35" s="12"/>
-      <c r="E35" s="8"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E35" s="24"/>
+      <c r="F35" s="8"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="12"/>
       <c r="C36" s="5"/>
       <c r="D36" s="12"/>
-      <c r="E36" s="8"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E36" s="24"/>
+      <c r="F36" s="8"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="12"/>
       <c r="C37" s="5"/>
       <c r="D37" s="12"/>
-      <c r="E37" s="8"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E37" s="24"/>
+      <c r="F37" s="8"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="12"/>
       <c r="C38" s="5"/>
       <c r="D38" s="12"/>
-      <c r="E38" s="8"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E38" s="24"/>
+      <c r="F38" s="8"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="12"/>
       <c r="C39" s="5"/>
       <c r="D39" s="12"/>
-      <c r="E39" s="8"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A40" s="2"/>
-      <c r="B40" s="12"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="12"/>
-      <c r="E40" s="8"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="8"/>
+    </row>
+    <row r="40" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="3"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="23"/>
+    </row>
+    <row r="41" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E41" s="28">
+        <f>SUM(E5:E12,E17:E40)</f>
+        <v>259.5</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E8" r:id="rId1" xr:uid="{D580C034-BEEA-46FA-B8C5-DFFDAC6C344A}"/>
-    <hyperlink ref="E9" r:id="rId2" xr:uid="{C39A8AD1-20D0-4B37-9511-742C314380FE}"/>
-    <hyperlink ref="E12" r:id="rId3" display="https://www.amazon.de/QUPERR-Sicherung-Akku-Adapter-Lithium-Akku-Power-Converter/dp/B0BPRYRGVF/ref=sr_1_6?__mk_de_DE=ÅMÅŽÕÑ&amp;crid=276VZBEJ40QUX&amp;dib=eyJ2IjoiMSJ9.7SKdXH7QLVLBjgwq-4cSCmbfxWZX8zEXSMFm1-XC4fKXJnAK8tr-OUUHGSCVjd96leUb2TzWPY70SoNDNuofOuOwgBoaw3QEOZNwy2e21XDrZdrocEDUCDjjEvyJknbExeVieTLSwac3dbVEVAA3MsZyqtxId76PBSZqhRb2NTPzAfUzjW1d9oUUEX1JwUPF_MGxOsbfKxQzeZp9oAaAs81eWJjCOFA_fS7nYSsUeDY.9tHZQNh8Hzu9MMm-HiRbNy1zVDuVNl88OwXy5J3tccM&amp;dib_tag=se&amp;keywords=makita+akku+schnittstelle&amp;qid=1747144685&amp;sprefix=makita+akku+schnittstell%2Caps%2C146&amp;sr=8-6" xr:uid="{C58E542C-DD92-4972-992C-AD26836DE70F}"/>
-    <hyperlink ref="E7" r:id="rId4" xr:uid="{0C4E5862-7CA3-4826-91A9-2BFF4E1C4344}"/>
+    <hyperlink ref="F8" r:id="rId1" xr:uid="{D580C034-BEEA-46FA-B8C5-DFFDAC6C344A}"/>
+    <hyperlink ref="F9" r:id="rId2" xr:uid="{C39A8AD1-20D0-4B37-9511-742C314380FE}"/>
+    <hyperlink ref="F12" r:id="rId3" display="https://www.amazon.de/QUPERR-Sicherung-Akku-Adapter-Lithium-Akku-Power-Converter/dp/B0BPRYRGVF/ref=sr_1_6?__mk_de_DE=ÅMÅŽÕÑ&amp;crid=276VZBEJ40QUX&amp;dib=eyJ2IjoiMSJ9.7SKdXH7QLVLBjgwq-4cSCmbfxWZX8zEXSMFm1-XC4fKXJnAK8tr-OUUHGSCVjd96leUb2TzWPY70SoNDNuofOuOwgBoaw3QEOZNwy2e21XDrZdrocEDUCDjjEvyJknbExeVieTLSwac3dbVEVAA3MsZyqtxId76PBSZqhRb2NTPzAfUzjW1d9oUUEX1JwUPF_MGxOsbfKxQzeZp9oAaAs81eWJjCOFA_fS7nYSsUeDY.9tHZQNh8Hzu9MMm-HiRbNy1zVDuVNl88OwXy5J3tccM&amp;dib_tag=se&amp;keywords=makita+akku+schnittstelle&amp;qid=1747144685&amp;sprefix=makita+akku+schnittstell%2Caps%2C146&amp;sr=8-6" xr:uid="{C58E542C-DD92-4972-992C-AD26836DE70F}"/>
+    <hyperlink ref="F7" r:id="rId4" xr:uid="{0C4E5862-7CA3-4826-91A9-2BFF4E1C4344}"/>
+    <hyperlink ref="F10" r:id="rId5" xr:uid="{332C0DDF-E49C-4815-A8CB-1575E2601414}"/>
+    <hyperlink ref="F17" r:id="rId6" xr:uid="{01BFAFB1-3B7D-48A8-BBB9-8125A53B1C2F}"/>
+    <hyperlink ref="F18" r:id="rId7" xr:uid="{97AD1438-0EB5-41F9-BB4F-526C6CECFC9B}"/>
+    <hyperlink ref="F19" r:id="rId8" xr:uid="{04A7E77E-F486-4058-B492-EC778840C9D6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>